<commit_message>
Round 5 + 6 measurements
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Fat_Muscle_Measurements.xlsx
+++ b/data/Fat_Muscle_Measurements.xlsx
@@ -12,7 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2nd Progress (20 Apr 26)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3rd Progress (5 May 26)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4th Progress (19 May 26)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5th Progress (8 Jun 26)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6th Progress (22 Jun 26)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2137,6 +2139,316 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Fat &amp; Muscle Campaign — 5th Progress Measurements (8 Jun 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Body Fat %</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Muscle %</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Maneenund</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="C3" t="n">
+        <v>58.3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pipat</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C4" t="n">
+        <v>75.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Pruang</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>76.40000000000001</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Orawan</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>59.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>66.90000000000001</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bob</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="C8" t="n">
+        <v>64.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ben</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="C9" t="n">
+        <v>69.90000000000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GROUP AVERAGE</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Fat &amp; Muscle Campaign — 6th Progress Measurements (22 Jun 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Body Fat %</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Muscle %</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ohm</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C3" t="n">
+        <v>60.6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pipat</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>76.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Pruang</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="C5" t="n">
+        <v>76.7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Nott</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="C6" t="n">
+        <v>73.2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Orawan</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>59.8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ann</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>72.40000000000001</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Piyathida</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>72.09999999999999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Bob</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="C10" t="n">
+        <v>64.09999999999999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ben</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="C11" t="n">
+        <v>70.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GROUP AVERAGE</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Final round (round 8) measurements; round 7 skipped
</commit_message>
<xml_diff>
--- a/data/Fat_Muscle_Measurements.xlsx
+++ b/data/Fat_Muscle_Measurements.xlsx
@@ -14,7 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4th Progress (19 May 26)" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5th Progress (8 Jun 26)" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6th Progress (22 Jun 26)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8th Progress (20 Jul 26)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2449,6 +2450,226 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Fat &amp; Muscle Campaign — 8th Progress Measurements (20 Jul 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Body Fat %</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Muscle %</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ohm</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>35.75</v>
+      </c>
+      <c r="C3" t="n">
+        <v>60.85</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Maneenund</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>58.75</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Pipat</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="C5" t="n">
+        <v>76.90000000000001</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pruang</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="C6" t="n">
+        <v>76.8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nott</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>73.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Orawan</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>36</v>
+      </c>
+      <c r="C8" t="n">
+        <v>60.2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Jue</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>29.05</v>
+      </c>
+      <c r="C9" t="n">
+        <v>67.15000000000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Ann</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="C10" t="n">
+        <v>72.2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Piyathida</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="C11" t="n">
+        <v>71.90000000000001</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Best</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="C12" t="n">
+        <v>71.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sonny</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="C13" t="n">
+        <v>74.09999999999999</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Bob</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>32</v>
+      </c>
+      <c r="C14" t="n">
+        <v>64.3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ben</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="C15" t="n">
+        <v>71.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GROUP AVERAGE</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>